<commit_message>
Added HW Premium 2 items
</commit_message>
<xml_diff>
--- a/inventory/Inventory.xlsx
+++ b/inventory/Inventory.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Hot Wheels Mainline" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1396" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1412" uniqueCount="368">
   <si>
     <t>Code</t>
   </si>
@@ -1114,6 +1114,18 @@
   </si>
   <si>
     <t>AMARU GTC</t>
+  </si>
+  <si>
+    <t>JKY01</t>
+  </si>
+  <si>
+    <t>2017 NISSAN GT-R (R35)</t>
+  </si>
+  <si>
+    <t>JKY27</t>
+  </si>
+  <si>
+    <t>CUSTOM/PERSONNALISÉ '70 HONDA N600</t>
   </si>
 </sst>
 </file>
@@ -1174,7 +1186,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1207,6 +1219,9 @@
     <xf numFmtId="14" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="17" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4711,10 +4726,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="4" max="4" width="43.5546875" customWidth="1"/>
+    <col min="5" max="5" width="21.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
@@ -4889,6 +4905,76 @@
         <v>11</v>
       </c>
       <c r="K5" s="18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="24" t="s">
+        <v>364</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="24" t="s">
+        <v>365</v>
+      </c>
+      <c r="E6" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="F6" s="25">
+        <v>46113</v>
+      </c>
+      <c r="G6" s="24">
+        <v>299</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="I6" s="26">
+        <v>399</v>
+      </c>
+      <c r="J6" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="K6" s="18" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="24" t="s">
+        <v>366</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="24" t="s">
+        <v>367</v>
+      </c>
+      <c r="E7" s="16" t="s">
+        <v>193</v>
+      </c>
+      <c r="F7" s="25">
+        <v>46143</v>
+      </c>
+      <c r="G7" s="24">
+        <v>299</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="26">
+        <v>399</v>
+      </c>
+      <c r="J7" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="K7" s="18" t="s">
         <v>10</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added convert.py to convert the excel inventory into json
</commit_message>
<xml_diff>
--- a/inventory/Inventory.xlsx
+++ b/inventory/Inventory.xlsx
@@ -4,12 +4,12 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" activeTab="1"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="1" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Hot Wheels Mainline" sheetId="1" r:id="rId1"/>
     <sheet name="Hot Wheels Premium" sheetId="2" r:id="rId2"/>
-    <sheet name="Hot Wheels Treaure Hunt" sheetId="3" r:id="rId3"/>
+    <sheet name="Hot Wheels Treasure Hunt" sheetId="3" r:id="rId3"/>
     <sheet name="Hot Wheels 5 Packs" sheetId="4" r:id="rId4"/>
     <sheet name="Matchbox Card" sheetId="5" r:id="rId5"/>
     <sheet name="Matchbox Box" sheetId="6" r:id="rId6"/>

</xml_diff>

<commit_message>
3 items SOLD - Matchbox Moving parts - Bundle & HW Premium
</commit_message>
<xml_diff>
--- a/inventory/Inventory.xlsx
+++ b/inventory/Inventory.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="1" activeTab="6"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="2" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Hot Wheels Mainline" sheetId="1" r:id="rId1"/>
@@ -4797,7 +4797,7 @@
         <v>699</v>
       </c>
       <c r="J2" s="18" t="s">
-        <v>11</v>
+        <v>116</v>
       </c>
       <c r="K2" s="18" t="s">
         <v>10</v>
@@ -7383,7 +7383,7 @@
         <v>609</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>11</v>
+        <v>116</v>
       </c>
       <c r="K2" s="7" t="s">
         <v>10</v>
@@ -8068,7 +8068,7 @@
         <v>1617</v>
       </c>
       <c r="J6" s="8" t="s">
-        <v>11</v>
+        <v>116</v>
       </c>
       <c r="K6" s="8" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
Matchbox Box McLaren F1 GT
</commit_message>
<xml_diff>
--- a/inventory/Inventory.xlsx
+++ b/inventory/Inventory.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016"/>
+    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016" firstSheet="2" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Hot Wheels Mainline" sheetId="1" r:id="rId1"/>
@@ -7084,7 +7084,7 @@
         <v>289</v>
       </c>
       <c r="J17" s="7" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K17" s="2" t="s">
         <v>10</v>
@@ -8927,7 +8927,7 @@
         <v>887</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>11</v>
+        <v>114</v>
       </c>
       <c r="K31" s="7" t="s">
         <v>10</v>

</xml_diff>